<commit_message>
Mise à jour Excel
</commit_message>
<xml_diff>
--- a/Documents/APP/20250916_dicovar_reflexion_e3n.xlsx
+++ b/Documents/APP/20250916_dicovar_reflexion_e3n.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49B2BF6-BE47-4F78-8F0B-3848E0E5BC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5D6390-F11A-4C35-9118-4C4DC05898B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5830,55 +5830,55 @@
     <t>Questionnaire Q13</t>
   </si>
   <si>
-    <t>Documents\APP\pdf\E3N_Q1.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q2.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q3_sante.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q3_alimentaire.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q4.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q5.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q6.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q7.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q8_sante.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q9.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q10.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q11.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q12.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E3N_Q13.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E4N-G1_Q1.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E4N-G1_Q2.pdf</t>
-  </si>
-  <si>
-    <t>Documents\APP\pdf\E4N-G1_Q3.pdf</t>
+    <t>Documents/APP/pdf/E3N_Q1.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q2.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q3_sante.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q3_alimentaire.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q4.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q5.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q6.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q7.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q8_sante.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q9.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q10.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q11.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q12.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E3N_Q13.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E4N-G1_Q1.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E4N-G1_Q2.pdf</t>
+  </si>
+  <si>
+    <t>Documents/APP/pdf/E4N-G1_Q3.pdf</t>
   </si>
 </sst>
 </file>
@@ -28403,7 +28403,7 @@
         <v>1827</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>1816</v>
       </c>
@@ -28426,7 +28426,7 @@
         <v>1828</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>1816</v>
       </c>

</xml_diff>